<commit_message>
Improve the visibility and styling of the download button and update session data
Update the download button styling in the PartnersManagement component to match existing button styles and correct the visibility issue. Additionally, update the 'updated_at' timestamp for multiple analytics sessions in the server data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/lhx8L0S
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -520,9 +520,68 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2025-10-14T18:08:00.835Z</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ELOIT</v>
+      </c>
+      <c r="D3" t="str">
+        <v>partner@photall.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>0651334512</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://photall.com</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2 rue de la Peyrolerie</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Capdenac</v>
+      </c>
+      <c r="I3" t="str">
+        <v>46100</v>
+      </c>
+      <c r="J3" t="str">
+        <v>FR</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Photo, Video, Film</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>No</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve download button styling and remove unnecessary text
Update the download button's appearance by adjusting its styling and remove a redundant French date format notification from the partner management section.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/lhx8L0S
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,68 +461,9 @@
         <v>Consent</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2025-10-14T18:21:27.715Z</v>
-      </c>
-      <c r="B2" t="str">
-        <v>ELOIT</v>
-      </c>
-      <c r="D2" t="str">
-        <v>contact@eloit.com</v>
-      </c>
-      <c r="E2" t="str">
-        <v>0651334512</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://eloit.com</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2 rue de la Peyrolerie</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Capdenac</v>
-      </c>
-      <c r="I2" t="str">
-        <v>46100</v>
-      </c>
-      <c r="J2" t="str">
-        <v>FR</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Photo, Video, Film</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v>No</v>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add language switcher to partner intake forms and fix scrolling
Implement a language switcher component on both English and French partner intake forms, allowing users to navigate between language versions. Also, ensure smooth scrolling to the top of the page after form submission.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/9yPT32I
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -458,68 +458,9 @@
         <v>Consent</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>2025-10-15T05:39:50.370Z</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Eloit</v>
-      </c>
-      <c r="C2" t="str">
-        <v>e@e.com</v>
-      </c>
-      <c r="D2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v>France</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Prints</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve partner intake form with corrected alignment and contact information
Update partner intake forms to fix checkbox alignment, modify French text for service selection, and add contact information with translated required fields.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/lxJmWIn
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -458,9 +458,71 @@
         <v>Consent</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2025-10-15T07:28:10.021Z</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ccccc</v>
+      </c>
+      <c r="C2" t="str">
+        <v>cc@dd.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0606</v>
+      </c>
+      <c r="F2" t="str">
+        <v>photall.com</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>France</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Prints</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve partner intake form and session data
Update partner intake forms for EN and FR locales with improved placeholder styling. Adjust session duration in analytics-sessions.json and add a new session entry.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/n6raCIC
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -520,9 +520,71 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2025-10-15T07:42:02.913Z</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ngoc boite</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ngoc@outlook.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E3" t="str">
+        <v>12346856263</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ngoc.com</v>
+      </c>
+      <c r="G3" t="str">
+        <v>123 rue abc</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Batiment BCB</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Capdenac</v>
+      </c>
+      <c r="J3" t="str">
+        <v>12345</v>
+      </c>
+      <c r="K3" t="str">
+        <v>France</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Polaroid/Instax, Negatives 35mm</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>8mm, Super 8</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v>Digital8, U-Matic, MiniDV</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>USB, DVD/Blu-ray</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change button text color for better visibility on partner form
Updates the "Sauvegarder les modifications" button text color to black from white for improved contrast against the gray background in the partner intake form.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/2QzUgKv
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -550,19 +550,19 @@
         <v>Yes</v>
       </c>
       <c r="V2" t="str">
-        <v>Pending</v>
+        <v>Approved</v>
       </c>
       <c r="W2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="X2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="Y2" t="str">
-        <v/>
+        <v>45.5186</v>
       </c>
       <c r="Z2" t="str">
-        <v/>
+        <v>1.9981</v>
       </c>
       <c r="AA2" t="str">
         <v>eloit-inc</v>

</xml_diff>

<commit_message>
Update partner directory filters and data to French
Refactor `PartnerDirectoryFR.tsx` to use French labels for service and format filters, and update coordinates for "Eloit Inc" in `public/partners.json`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/2QzUgKv
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -559,10 +559,10 @@
         <v>TRUE</v>
       </c>
       <c r="Y2" t="str">
-        <v>45.5186</v>
+        <v>44.581099038048706</v>
       </c>
       <c r="Z2" t="str">
-        <v>1.9981</v>
+        <v>2.070213083026406</v>
       </c>
       <c r="AA2" t="str">
         <v>eloit-inc</v>

</xml_diff>

<commit_message>
Update partner directory to display only map-visible partners
Refactors PartnerDirectoryFR.tsx to use mappablePartners instead of filteredPartners, ensuring only partners currently visible on the map are listed. Adds new partner data to public/partners.json.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/2QzUgKv
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -568,9 +568,175 @@
         <v>eloit-inc</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2025-10-15T15:08:24.643Z</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lebolabo</v>
+      </c>
+      <c r="C3" t="str">
+        <v>test@lebolabo.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E3" t="str">
+        <v>+33 6 51 33 12</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://lebolabo.com/</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2 rue de la Soif</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>Bordeaux</v>
+      </c>
+      <c r="J3" t="str">
+        <v>46130</v>
+      </c>
+      <c r="K3" t="str">
+        <v>France</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Prints, Albums</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>USB</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v>Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W3" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="X3" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v>lebolabo</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2025-10-15T15:14:23.310Z</v>
+      </c>
+      <c r="B4" t="str">
+        <v>NGOC TEST</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ngoc@test.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E4" t="str">
+        <v>12 65 25 15 45</v>
+      </c>
+      <c r="F4" t="str">
+        <v>test.com</v>
+      </c>
+      <c r="G4" t="str">
+        <v>68 Av. Jean Jaurès</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Souillac</v>
+      </c>
+      <c r="J4" t="str">
+        <v>46200</v>
+      </c>
+      <c r="K4" t="str">
+        <v>France</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Prints, Negatives 35mm</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>8mm, Super 8</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v>VHS, MiniDV, Digital8</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>USB, DVD/Blu-ray</v>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v>description test</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="V4" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="W4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>44.9046780724082</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>1.4671430115554622</v>
+      </c>
+      <c r="AA4" t="str">
+        <v>ngoc-test</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change text color on partner intake form to improve visibility
Update CSS styles for the partner intake form to ensure text is black on a gray background.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/k9AwiTu
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,88 +397,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AC4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Timestamp</v>
       </c>
       <c r="B1" t="str">
+        <v>Partner Type</v>
+      </c>
+      <c r="C1" t="str">
         <v>Partner Name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Email</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Email_Public</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Phone</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>Phone_Public</v>
+      </c>
+      <c r="H1" t="str">
         <v>Website</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Address</v>
       </c>
-      <c r="H1" t="str">
-        <v>Complément d'adresse</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
+        <v>Address Line 2</v>
+      </c>
+      <c r="K1" t="str">
         <v>City</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Postal Code</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Country</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Photo Formats</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Other Photo</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>Film Formats</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Other Film</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>Video Cassettes</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>Other Video</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>Delivery</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>Other Delivery</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Public Description</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Consent</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
         <v>Status</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Y1" t="str">
         <v>Is_Active</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Z1" t="str">
         <v>Show_On_Map</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AA1" t="str">
         <v>lat</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AB1" t="str">
         <v>lng</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AC1" t="str">
         <v>slug</v>
       </c>
     </row>
@@ -487,84 +493,90 @@
         <v>2025-10-15T10:16:29.295Z</v>
       </c>
       <c r="B2" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C2" t="str">
         <v>Eloit Inc</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>stephane@eloit.com</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>+33 6 51 33 45 12</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H2" t="str">
         <v>photall.com</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>2 rue de la Peyrolerie</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>Capdenac</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>46130</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>France</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>Prints, Negatives 35mm, Slides 35mm, Medium format 120/220</v>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>Super 8, 8mm</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v>Betamax, VHS, Digital8</v>
       </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
         <v>USB, External drive</v>
       </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str" xml:space="preserve">
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str" xml:space="preserve">
         <v xml:space="preserve">La solution idéale pour sauvegarder vos souvenirs et les visionner facilement !
 Utilisation de scanners professionnels.
 Correction colorimétrique des diapositives scannées afin d’améliorer le rendu des couleurs et minimiser les – dégâts du temps.
 Optimisation des contrastes et de l’exposition afin d’adapter les images à une consultation sur un écran d’ordinateur ou de TV (le contraste et l’exposition sont initialement prévus pour une projection sur écran avec une ampoule à forte intensité).</v>
       </c>
-      <c r="U2" t="str">
+      <c r="W2" t="str">
         <v>Yes</v>
       </c>
-      <c r="V2" t="str">
+      <c r="X2" t="str">
         <v>Approved</v>
       </c>
-      <c r="W2" t="str">
+      <c r="Y2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="X2" t="str">
+      <c r="Z2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="AA2" t="str">
         <v>44.581099038048706</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AB2" t="str">
         <v>2.070213083026406</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AC2" t="str">
         <v>eloit-inc</v>
       </c>
     </row>
@@ -573,44 +585,44 @@
         <v>2025-10-15T15:08:24.643Z</v>
       </c>
       <c r="B3" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C3" t="str">
         <v>Lebolabo</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>test@lebolabo.com</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>+33 6 51 33 12</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H3" t="str">
         <v>https://lebolabo.com/</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>2 rue de la Soif</v>
       </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>Bordeaux</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v>46130</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>France</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>Prints, Albums</v>
       </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
       <c r="O3" t="str">
         <v/>
       </c>
@@ -621,33 +633,39 @@
         <v/>
       </c>
       <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
         <v>USB</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
-      <c r="T3" t="str">
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
         <v>Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>Yes</v>
       </c>
-      <c r="V3" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="W3" t="str">
+      <c r="X3" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y3" t="str">
         <v>FALSE</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Z3" t="str">
         <v>FALSE</v>
       </c>
-      <c r="Y3" t="str">
-        <v/>
-      </c>
-      <c r="Z3" t="str">
-        <v/>
-      </c>
       <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
         <v>lebolabo</v>
       </c>
     </row>
@@ -656,87 +674,93 @@
         <v>2025-10-15T15:14:23.310Z</v>
       </c>
       <c r="B4" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C4" t="str">
         <v>NGOC TEST</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>ngoc@test.com</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>12 65 25 15 45</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H4" t="str">
         <v>test.com</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>68 Av. Jean Jaurès</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>Souillac</v>
       </c>
-      <c r="J4" t="str">
+      <c r="L4" t="str">
         <v>46200</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>France</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>Prints, Negatives 35mm</v>
       </c>
-      <c r="M4" t="str">
-        <v/>
-      </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>8mm, Super 8</v>
       </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
         <v>VHS, MiniDV, Digital8</v>
       </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
         <v>USB, DVD/Blu-ray</v>
       </c>
-      <c r="S4" t="str">
-        <v/>
-      </c>
-      <c r="T4" t="str">
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
         <v>description test</v>
       </c>
-      <c r="U4" t="str">
+      <c r="W4" t="str">
         <v>Yes</v>
       </c>
-      <c r="V4" t="str">
+      <c r="X4" t="str">
         <v>Approved</v>
       </c>
-      <c r="W4" t="str">
+      <c r="Y4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="X4" t="str">
+      <c r="Z4" t="str">
         <v>TRUE</v>
       </c>
-      <c r="Y4" t="str">
+      <c r="AA4" t="str">
         <v>44.9046780724082</v>
       </c>
-      <c r="Z4" t="str">
+      <c r="AB4" t="str">
         <v>1.4671430115554622</v>
       </c>
-      <c r="AA4" t="str">
+      <c r="AC4" t="str">
         <v>ngoc-test</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve partner intake form validation and data handling
Update partner submission handling with enhanced Zod schema validation and React Hook Form integration.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/DWH7y8c
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC4"/>
+  <dimension ref="A1:AC3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,39 +488,39 @@
         <v>slug</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2025-10-15T10:16:29.295Z</v>
+        <v>2025-10-15T15:08:24.643Z</v>
       </c>
       <c r="B2" t="str">
         <v>digitization</v>
       </c>
       <c r="C2" t="str">
-        <v>Eloit Inc</v>
+        <v>Lebolabo</v>
       </c>
       <c r="D2" t="str">
-        <v>stephane@eloit.com</v>
+        <v>test@lebolabo.com</v>
       </c>
       <c r="E2" t="str">
         <v>TRUE</v>
       </c>
       <c r="F2" t="str">
-        <v>+33 6 51 33 45 12</v>
+        <v>+33 6 51 33 12</v>
       </c>
       <c r="G2" t="str">
         <v>FALSE</v>
       </c>
       <c r="H2" t="str">
-        <v>photall.com</v>
+        <v>https://lebolabo.com/</v>
       </c>
       <c r="I2" t="str">
-        <v>2 rue de la Peyrolerie</v>
+        <v>2 rue de la Soif</v>
       </c>
       <c r="J2" t="str">
         <v/>
       </c>
       <c r="K2" t="str">
-        <v>Capdenac</v>
+        <v>Bordeaux</v>
       </c>
       <c r="L2" t="str">
         <v>46130</v>
@@ -529,123 +529,120 @@
         <v>France</v>
       </c>
       <c r="N2" t="str">
-        <v>Prints, Negatives 35mm, Slides 35mm, Medium format 120/220</v>
+        <v>Prints, Albums</v>
       </c>
       <c r="O2" t="str">
         <v/>
       </c>
       <c r="P2" t="str">
-        <v>Super 8, 8mm</v>
+        <v/>
       </c>
       <c r="Q2" t="str">
         <v/>
       </c>
       <c r="R2" t="str">
-        <v>Betamax, VHS, Digital8</v>
+        <v/>
       </c>
       <c r="S2" t="str">
         <v/>
       </c>
       <c r="T2" t="str">
-        <v>USB, External drive</v>
+        <v>USB</v>
       </c>
       <c r="U2" t="str">
         <v/>
       </c>
-      <c r="V2" t="str" xml:space="preserve">
-        <v xml:space="preserve">La solution idéale pour sauvegarder vos souvenirs et les visionner facilement !
-Utilisation de scanners professionnels.
-Correction colorimétrique des diapositives scannées afin d’améliorer le rendu des couleurs et minimiser les – dégâts du temps.
-Optimisation des contrastes et de l’exposition afin d’adapter les images à une consultation sur un écran d’ordinateur ou de TV (le contraste et l’exposition sont initialement prévus pour une projection sur écran avec une ampoule à forte intensité).</v>
+      <c r="V2" t="str">
+        <v>Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
       </c>
       <c r="W2" t="str">
         <v>Yes</v>
       </c>
       <c r="X2" t="str">
-        <v>Pending</v>
+        <v>Approved</v>
       </c>
       <c r="Y2" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="Z2" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AA2" t="str">
-        <v>44.581099038048706</v>
+        <v/>
       </c>
       <c r="AB2" t="str">
-        <v>2.070213083026406</v>
+        <v/>
       </c>
       <c r="AC2" t="str">
-        <v>eloit-inc</v>
+        <v>lebolabo</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-10-15T15:08:24.643Z</v>
+        <v>2025-10-15T15:14:23.310Z</v>
       </c>
       <c r="B3" t="str">
         <v>digitization</v>
       </c>
       <c r="C3" t="str">
-        <v>Lebolabo</v>
+        <v>NGOC TEST</v>
       </c>
       <c r="D3" t="str">
-        <v>test@lebolabo.com</v>
+        <v>ngoc@test.com</v>
       </c>
       <c r="E3" t="str">
         <v>TRUE</v>
       </c>
       <c r="F3" t="str">
-        <v>+33 6 51 33 12</v>
+        <v>12 65 25 15 45</v>
       </c>
       <c r="G3" t="str">
         <v>FALSE</v>
       </c>
       <c r="H3" t="str">
-        <v>https://lebolabo.com/</v>
+        <v>test.com</v>
       </c>
       <c r="I3" t="str">
-        <v>2 rue de la Soif</v>
+        <v>68 Av. Jean Jaurès</v>
       </c>
       <c r="J3" t="str">
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>Bordeaux</v>
+        <v>Souillac</v>
       </c>
       <c r="L3" t="str">
-        <v>46130</v>
+        <v>46200</v>
       </c>
       <c r="M3" t="str">
         <v>France</v>
       </c>
       <c r="N3" t="str">
-        <v>Prints, Albums</v>
+        <v>Prints, Negatives 35mm</v>
       </c>
       <c r="O3" t="str">
         <v/>
       </c>
       <c r="P3" t="str">
-        <v/>
+        <v>8mm, Super 8</v>
       </c>
       <c r="Q3" t="str">
         <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>VHS, MiniDV, Digital8</v>
       </c>
       <c r="S3" t="str">
         <v/>
       </c>
       <c r="T3" t="str">
-        <v>USB</v>
+        <v>USB, DVD/Blu-ray</v>
       </c>
       <c r="U3" t="str">
         <v/>
       </c>
       <c r="V3" t="str">
-        <v>Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
+        <v>description test</v>
       </c>
       <c r="W3" t="str">
         <v>Yes</v>
@@ -654,113 +651,24 @@
         <v>Approved</v>
       </c>
       <c r="Y3" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="Z3" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="AA3" t="str">
-        <v/>
+        <v>44.9046780724082</v>
       </c>
       <c r="AB3" t="str">
-        <v/>
+        <v>1.4671430115554622</v>
       </c>
       <c r="AC3" t="str">
-        <v>lebolabo</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2025-10-15T15:14:23.310Z</v>
-      </c>
-      <c r="B4" t="str">
-        <v>digitization</v>
-      </c>
-      <c r="C4" t="str">
-        <v>NGOC TEST</v>
-      </c>
-      <c r="D4" t="str">
-        <v>ngoc@test.com</v>
-      </c>
-      <c r="E4" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="F4" t="str">
-        <v>12 65 25 15 45</v>
-      </c>
-      <c r="G4" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="H4" t="str">
-        <v>test.com</v>
-      </c>
-      <c r="I4" t="str">
-        <v>68 Av. Jean Jaurès</v>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
-        <v>Souillac</v>
-      </c>
-      <c r="L4" t="str">
-        <v>46200</v>
-      </c>
-      <c r="M4" t="str">
-        <v>France</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Prints, Negatives 35mm</v>
-      </c>
-      <c r="O4" t="str">
-        <v/>
-      </c>
-      <c r="P4" t="str">
-        <v>8mm, Super 8</v>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
-        <v>VHS, MiniDV, Digital8</v>
-      </c>
-      <c r="S4" t="str">
-        <v/>
-      </c>
-      <c r="T4" t="str">
-        <v>USB, DVD/Blu-ray</v>
-      </c>
-      <c r="U4" t="str">
-        <v/>
-      </c>
-      <c r="V4" t="str">
-        <v>description test</v>
-      </c>
-      <c r="W4" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="X4" t="str">
-        <v>Approved</v>
-      </c>
-      <c r="Y4" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Z4" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="AA4" t="str">
-        <v>44.9046780724082</v>
-      </c>
-      <c r="AB4" t="str">
-        <v>1.4671430115554622</v>
-      </c>
-      <c r="AC4" t="str">
         <v>ngoc-test</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add a link to view partner map from the menu
Import `ExternalLink` icon and add a new button to `PartnersManagementEnhanced` component to open the partner map in a new tab. Remove an existing partner entry from `public/partners.json`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/DWH7y8c
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -666,9 +666,98 @@
         <v>ngoc-test</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2025-10-15T17:06:52.030Z</v>
+      </c>
+      <c r="B4" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C4" t="str">
+        <v>eeeee</v>
+      </c>
+      <c r="D4" t="str">
+        <v>sss2ooe@ddd.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H4" t="str">
+        <v>ddd.com</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>Prints</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>Digital8</v>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v>External drive, USB</v>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v>ddd.comddd.comddd.comddd.comddd.com</v>
+      </c>
+      <c r="W4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X4" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="AA4">
+        <v>44.44543449469977</v>
+      </c>
+      <c r="AB4">
+        <v>1.4452141176732154</v>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add timestamp to partner intake form data for better tracking
Update Partner interface to include a timestamp field and modify partner-submissions.xlsx.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/DWH7y8c
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -567,11 +567,11 @@
       <c r="Z2" t="str">
         <v>FALSE</v>
       </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
+      <c r="AA2">
+        <v>30.4</v>
+      </c>
+      <c r="AB2">
+        <v>1.5</v>
       </c>
       <c r="AC2" t="str">
         <v>lebolabo</v>

</xml_diff>

<commit_message>
Update partner intake form with improved input validation and privacy
Add improved input validation and privacy controls to the partner intake form.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/DWH7y8c
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -514,7 +514,7 @@
         <v>https://lebolabo.com/</v>
       </c>
       <c r="I2" t="str">
-        <v>2 rue de la Soif</v>
+        <v>48 Rue Bergeret</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -523,7 +523,7 @@
         <v>Bordeaux</v>
       </c>
       <c r="L2" t="str">
-        <v>46130</v>
+        <v>33000</v>
       </c>
       <c r="M2" t="str">
         <v>France</v>
@@ -568,10 +568,10 @@
         <v>FALSE</v>
       </c>
       <c r="AA2">
-        <v>30.4</v>
+        <v>44.831897557776564</v>
       </c>
       <c r="AB2">
-        <v>1.5</v>
+        <v>-0.5678587426661484</v>
       </c>
       <c r="AC2" t="str">
         <v>lebolabo</v>

</xml_diff>

<commit_message>
Update partner data and session duration for analytics
Add a new partner entry to public/partners.json and increase the duration for an analytics session in server/data/analytics-sessions.json.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/9VHpuRa
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -508,7 +508,7 @@
         <v>+33 6 51 33 12</v>
       </c>
       <c r="G2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="H2" t="str">
         <v>https://lebolabo.com/</v>
@@ -562,10 +562,10 @@
         <v>Approved</v>
       </c>
       <c r="Y2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="Z2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="AA2">
         <v>44.831897557776564</v>

</xml_diff>

<commit_message>
Update partner descriptions and session durations
Update the `public_description` for the "lebolabo" partner in `public/partners.json` and modify the `duration` and `updated_at` fields for a session in `server/data/analytics-sessions.json`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/9VHpuRa
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -488,7 +488,7 @@
         <v>slug</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>2025-10-15T15:08:24.643Z</v>
       </c>
@@ -552,8 +552,9 @@
       <c r="U2" t="str">
         <v/>
       </c>
-      <c r="V2" t="str">
-        <v>Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
+      <c r="V2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.
+Lebolabo réalise des numérisations photo par lot en basse résolution afin que vous puissiez visualiser vos images facilement sur un appareil numérique tel qu’un écran d’ordinateur, une tablette ou un smartphone (IPhone ou Android) et à moindre coût.</v>
       </c>
       <c r="W2" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
Add partner data for Switzerland, France, and Canada
Adds new partner entries to `public/partners.json` and updates mock analytics session data in `server/data/analytics-sessions.json` to include entries for Switzerland, France, and Canada.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/1mODD9b
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC4"/>
+  <dimension ref="A1:AC14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -756,9 +756,899 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2025-10-16T08:13:22.805Z</v>
+      </c>
+      <c r="B5" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Swiss Memory Lab</v>
+      </c>
+      <c r="D5" t="str">
+        <v>contact@swissmemorylab.ch</v>
+      </c>
+      <c r="E5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F5" t="str">
+        <v>+41 22 345 6789</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H5" t="str">
+        <v>swissmemorylab.ch</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Rue du Rhône 45</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>Geneva</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1204</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Switzerland</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Prints, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>Super 8, 16mm</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v>VHS, MiniDV</v>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v>In-person, Mail</v>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v>Spécialiste de la numérisation de médias depuis 1995. Nous offrons des services professionnels de haute qualité pour préserver vos souvenirs les plus précieux.</v>
+      </c>
+      <c r="W5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X5" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA5" t="str">
+        <v>46.2044</v>
+      </c>
+      <c r="AB5" t="str">
+        <v>6.1432</v>
+      </c>
+      <c r="AC5" t="str">
+        <v>swiss-memory-lab</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2025-10-16T08:13:24.713Z</v>
+      </c>
+      <c r="B6" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Zurich Digital Archives</v>
+      </c>
+      <c r="D6" t="str">
+        <v>info@zurichdigital.ch</v>
+      </c>
+      <c r="E6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F6" t="str">
+        <v>+41 44 123 4567</v>
+      </c>
+      <c r="G6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H6" t="str">
+        <v>zurichdigital.ch</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Bahnhofstrasse 100</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>Zurich</v>
+      </c>
+      <c r="L6" t="str">
+        <v>8001</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Switzerland</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Prints, Albums, Negatives 35mm</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v>8mm, Super 8</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v>VHS, Betamax, MiniDV</v>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v>In-person, Digital download</v>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v>Service de numérisation professionnel au cœur de Zurich. Technologie de pointe pour des résultats exceptionnels.</v>
+      </c>
+      <c r="W6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X6" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA6" t="str">
+        <v>47.3769</v>
+      </c>
+      <c r="AB6" t="str">
+        <v>8.5417</v>
+      </c>
+      <c r="AC6" t="str">
+        <v>zurich-digital-archives</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2025-10-16T08:13:26.457Z</v>
+      </c>
+      <c r="B7" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Lausanne Photo Scan</v>
+      </c>
+      <c r="D7" t="str">
+        <v>contact@lausannephotoscan.ch</v>
+      </c>
+      <c r="E7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F7" t="str">
+        <v>+41 21 987 6543</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H7" t="str">
+        <v>lausannephotoscan.ch</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Avenue de la Gare 15</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>Lausanne</v>
+      </c>
+      <c r="L7" t="str">
+        <v>1003</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Switzerland</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Prints, Slides 35mm</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v>Super 8</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v>Mail, Digital download</v>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v>Expert en numérisation de photos et films argentiques. Service rapide et soigné pour tous vos projets de préservation.</v>
+      </c>
+      <c r="W7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X7" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA7" t="str">
+        <v>46.5197</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>6.6323</v>
+      </c>
+      <c r="AC7" t="str">
+        <v>lausanne-photo-scan</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2025-10-16T08:13:28.921Z</v>
+      </c>
+      <c r="B8" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Brussels Heritage Digital</v>
+      </c>
+      <c r="D8" t="str">
+        <v>info@brusselsheritage.be</v>
+      </c>
+      <c r="E8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F8" t="str">
+        <v>+32 2 555 1234</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H8" t="str">
+        <v>brusselsheritage.be</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Boulevard Anspach 50</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>Brussels</v>
+      </c>
+      <c r="L8" t="str">
+        <v>1000</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Belgium</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Prints, Albums, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v>8mm, Super 8, 16mm</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v>VHS, VHS-C, MiniDV</v>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v>In-person, Mail, Digital download</v>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v>Centre de numérisation professionnel à Bruxelles. Plus de 20 ans d expertise dans la préservation de vos souvenirs familiaux.</v>
+      </c>
+      <c r="W8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X8" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>50.8503</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>4.3517</v>
+      </c>
+      <c r="AC8" t="str">
+        <v>brussels-heritage-digital</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2025-10-16T08:13:33.037Z</v>
+      </c>
+      <c r="B9" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Antwerp Media Transfer</v>
+      </c>
+      <c r="D9" t="str">
+        <v>contact@antwerpmt.be</v>
+      </c>
+      <c r="E9" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="F9" t="str">
+        <v>+32 3 789 4561</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H9" t="str">
+        <v>antwerpmt.be</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Meir 85</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>Antwerp</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2000</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Belgium</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Prints, Negatives 35mm</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v>Super 8</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v>VHS, Betamax, Digital8</v>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v>In-person, Mail</v>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v>Spécialiste de la conversion vidéo et photo à Anvers. Qualité professionnelle garantie pour tous vos médias anciens.</v>
+      </c>
+      <c r="W9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X9" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA9" t="str">
+        <v>51.2194</v>
+      </c>
+      <c r="AB9" t="str">
+        <v>4.4025</v>
+      </c>
+      <c r="AC9" t="str">
+        <v>antwerp-media-transfer</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2025-10-16T08:13:36.904Z</v>
+      </c>
+      <c r="B10" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Lyon Mémoire Numérique</v>
+      </c>
+      <c r="D10" t="str">
+        <v>contact@lyonmemoire.fr</v>
+      </c>
+      <c r="E10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F10" t="str">
+        <v>+33 4 78 56 34 12</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H10" t="str">
+        <v>lyonmemoire.fr</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Place Bellecour 12</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>Lyon</v>
+      </c>
+      <c r="L10" t="str">
+        <v>69002</v>
+      </c>
+      <c r="M10" t="str">
+        <v>France</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Prints, Albums, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v>8mm, Super 8</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v>VHS, MiniDV</v>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v>In-person, Mail, Digital download</v>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v>Votre expert en numérisation à Lyon. Service personnalisé et professionnel pour préserver vos précieux souvenirs de famille.</v>
+      </c>
+      <c r="W10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X10" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA10" t="str">
+        <v>45.7640</v>
+      </c>
+      <c r="AB10" t="str">
+        <v>4.8357</v>
+      </c>
+      <c r="AC10" t="str">
+        <v>lyon-memoire-numerique</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2025-10-16T08:13:41.049Z</v>
+      </c>
+      <c r="B11" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Marseille Photo Lab</v>
+      </c>
+      <c r="D11" t="str">
+        <v>info@marseillephotolab.fr</v>
+      </c>
+      <c r="E11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F11" t="str">
+        <v>+33 4 91 23 45 67</v>
+      </c>
+      <c r="G11" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="H11" t="str">
+        <v>marseillephotolab.fr</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Vieux-Port, Quai du Port 30</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>Marseille</v>
+      </c>
+      <c r="L11" t="str">
+        <v>13002</v>
+      </c>
+      <c r="M11" t="str">
+        <v>France</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Prints, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v>Super 8, 16mm</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v>VHS</v>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v>In-person, Digital download</v>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v>Laboratoire photo professionnel au cœur de Marseille. Numérisation haute résolution de vos photos, négatifs et films.</v>
+      </c>
+      <c r="W11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X11" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z11" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA11" t="str">
+        <v>43.2965</v>
+      </c>
+      <c r="AB11" t="str">
+        <v>5.3698</v>
+      </c>
+      <c r="AC11" t="str">
+        <v>marseille-photo-lab</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2025-10-16T08:13:44.824Z</v>
+      </c>
+      <c r="B12" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Nice Riviera Scan</v>
+      </c>
+      <c r="D12" t="str">
+        <v>contact@nicerivierascan.fr</v>
+      </c>
+      <c r="E12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F12" t="str">
+        <v>+33 4 93 87 65 43</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H12" t="str">
+        <v>nicerivierascan.fr</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Promenade des Anglais 45</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>Nice</v>
+      </c>
+      <c r="L12" t="str">
+        <v>06000</v>
+      </c>
+      <c r="M12" t="str">
+        <v>France</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Prints, Albums</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v>8mm, Super 8</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v>VHS, MiniDV, Digital8</v>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v>Mail, Digital download</v>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v>Service de numérisation sur la Côte d Azur. Qualité premium pour vos films et photos de vacances et souvenirs familiaux.</v>
+      </c>
+      <c r="W12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X12" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA12" t="str">
+        <v>43.7102</v>
+      </c>
+      <c r="AB12" t="str">
+        <v>7.2620</v>
+      </c>
+      <c r="AC12" t="str">
+        <v>nice-riviera-scan</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2025-10-16T08:13:49.096Z</v>
+      </c>
+      <c r="B13" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Montréal Film &amp; Photo</v>
+      </c>
+      <c r="D13" t="str">
+        <v>info@montrealfilm.ca</v>
+      </c>
+      <c r="E13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F13" t="str">
+        <v>+1 514 555 1234</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H13" t="str">
+        <v>montrealfilm.ca</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Rue Sainte-Catherine 1500</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>Montreal</v>
+      </c>
+      <c r="L13" t="str">
+        <v>H3G 1M8</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Prints, Albums, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v>8mm, Super 8, 16mm</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v>VHS, VHS-C, Betamax, MiniDV</v>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v>In-person, Mail, Digital download</v>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v>Expert en numérisation à Montréal depuis 15 ans. Service bilingue pour vos photos, films et vidéos de famille.</v>
+      </c>
+      <c r="W13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X13" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z13" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA13" t="str">
+        <v>45.5017</v>
+      </c>
+      <c r="AB13" t="str">
+        <v>-73.5673</v>
+      </c>
+      <c r="AC13" t="str">
+        <v>montreal-film-photo</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2025-10-16T08:13:53.460Z</v>
+      </c>
+      <c r="B14" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Toronto Memory Preservation</v>
+      </c>
+      <c r="D14" t="str">
+        <v>contact@torontomemory.ca</v>
+      </c>
+      <c r="E14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F14" t="str">
+        <v>+1 416 555 7890</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H14" t="str">
+        <v>torontomemory.ca</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Yonge Street 789</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Toronto</v>
+      </c>
+      <c r="L14" t="str">
+        <v>M5B 1Y8</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Prints, Negatives 35mm, Slides 35mm</v>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v>Super 8</v>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v>VHS, MiniDV, Digital8</v>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v>In-person, Mail, Digital download</v>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v>Professional digitization services in Toronto. We preserve your family memories with state-of-the-art technology and care.</v>
+      </c>
+      <c r="W14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X14" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z14" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA14" t="str">
+        <v>43.6532</v>
+      </c>
+      <c r="AB14" t="str">
+        <v>-79.3832</v>
+      </c>
+      <c r="AC14" t="str">
+        <v>toronto-memory-preservation</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update partner information with new locations and contact details
Modify the public/partners.json file to reflect updated location, contact details, and descriptions for several partners, including "NGOC TEST" and "lebolabo".

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/EDzbtB2
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -598,22 +598,22 @@
         <v>12 65 25 15 45</v>
       </c>
       <c r="G3" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="H3" t="str">
         <v>test.com</v>
       </c>
       <c r="I3" t="str">
-        <v>68 Av. Jean Jaurès</v>
+        <v>39 Rue Bergeret</v>
       </c>
       <c r="J3" t="str">
         <v/>
       </c>
       <c r="K3" t="str">
-        <v>Souillac</v>
+        <v>Bordeaux</v>
       </c>
       <c r="L3" t="str">
-        <v>46200</v>
+        <v/>
       </c>
       <c r="M3" t="str">
         <v>France</v>
@@ -657,11 +657,11 @@
       <c r="Z3" t="str">
         <v>TRUE</v>
       </c>
-      <c r="AA3" t="str">
-        <v>44.9046780724082</v>
-      </c>
-      <c r="AB3" t="str">
-        <v>1.4671430115554622</v>
+      <c r="AA3">
+        <v>44.82961</v>
+      </c>
+      <c r="AB3">
+        <v>-0.56748</v>
       </c>
       <c r="AC3" t="str">
         <v>ngoc-test</v>

</xml_diff>

<commit_message>
Add new partners to the partner directory and intake form
Updated the partner submission data with two new entries, ensuring schema consistency.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/EDzbtB2
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -658,10 +658,10 @@
         <v>TRUE</v>
       </c>
       <c r="AA3">
-        <v>44.82961</v>
+        <v>44.83179963473438</v>
       </c>
       <c r="AB3">
-        <v>-0.56748</v>
+        <v>-0.5680008374633064</v>
       </c>
       <c r="AC3" t="str">
         <v>ngoc-test</v>

</xml_diff>

<commit_message>
Add TSV upload option for partner submissions
Add a new TSV file upload option to the partner submission form for batch partner data entry.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/365df2cf-1884-444c-a9e8-235602456363/02a0c0b6-d5f3-47ec-a3d8-7138e4ba3033/EDzbtB2
</commit_message>
<xml_diff>
--- a/partner-submissions.xlsx
+++ b/partner-submissions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC14"/>
+  <dimension ref="A1:AC16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1646,9 +1646,187 @@
         <v>toronto-memory-preservation</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2025-10-15T09:34:01.258Z</v>
+      </c>
+      <c r="B15" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Photolix</v>
+      </c>
+      <c r="D15" t="str">
+        <v>lyon@photolix.fr</v>
+      </c>
+      <c r="E15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F15" t="str">
+        <v>04 78 89 33 13</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H15" t="str">
+        <v>www.photolix.fr</v>
+      </c>
+      <c r="I15" t="str">
+        <v>65 cours Vitton</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Lyon</v>
+      </c>
+      <c r="L15" t="str">
+        <v>69006</v>
+      </c>
+      <c r="M15" t="str">
+        <v>France</v>
+      </c>
+      <c r="N15" t="str">
+        <v>"Negatives 35mm, Medium format 120/220, Polaroid/Instax, Prints, Slides 35mm, Large format"</v>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v>"8mm, 9.5mm Pathé, Super 8, 16mm"</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v>"VHS, Video8/Hi8, MiniDV, DVCAM, Digital8, VHS-C, Betamax, U-Matic"</v>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v>"USB, Download link, DVD/Blu-ray"</v>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X15" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+      <c r="AC15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2025-10-16T10:07:29.740Z</v>
+      </c>
+      <c r="B16" t="str">
+        <v>digitization</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PANAJOU</v>
+      </c>
+      <c r="D16" t="str">
+        <v>contact@panajou.fr</v>
+      </c>
+      <c r="E16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="F16" t="str">
+        <v>+33556442269</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="H16" t="str">
+        <v>https://www.panajou.fr/</v>
+      </c>
+      <c r="I16" t="str">
+        <v>32 allées de Tourny</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>BORDEAUX</v>
+      </c>
+      <c r="L16" t="str">
+        <v>33000</v>
+      </c>
+      <c r="M16" t="str">
+        <v>France</v>
+      </c>
+      <c r="N16" t="str">
+        <v>"Prints, Albums, Negatives 35mm, Medium format 120/220, Slides 35mm, Large format, Polaroid/Instax"</v>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v>"8mm, 9.5mm Pathé, Super 8, 16mm"</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v>"VHS, Video8/Hi8, MiniDV, DVCAM, VHS-C, Digital8"</v>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v>USB</v>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="X16" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="Y16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="Z16" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+      <c r="AC16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>